<commit_message>
Correct quote export task status
The quote workflow exports XLSX and supports customer email, so the PDF wording left a completed task marked partial. Align both workbook views with Excel export and mark the item done.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4032,20 +4032,18 @@
       <c r="E31" s="49"/>
     </row>
     <row r="32">
-      <c r="A32" s="44" t="s">
-        <v>157</v>
+      <c r="A32" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Xuất file Excel / Gửi khách hàng</t>
+        </is>
       </c>
       <c r="B32" s="37" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C32" s="37"/>
-      <c r="D32" s="48" t="inlineStr">
-        <is>
-          <t>Thiếu xuất PDF báo giá; đã có XLSX và gửi email có preview.</t>
-        </is>
-      </c>
+      <c r="D32" s="48"/>
       <c r="E32" s="49"/>
     </row>
     <row r="33">
@@ -11726,7 +11724,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1">
+    <row r="11">
       <c r="A11" s="17">
         <v>10.0</v>
       </c>
@@ -11735,18 +11733,18 @@
       <c r="D11" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="F11" s="103" t="inlineStr">
-        <is>
-          <t>Detail page | Thiếu xuất PDF báo giá; đã có XLSX và gửi khách hàng có preview.</t>
-        </is>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>Thông tin báo giá, version, duyệt nội bộ, in/xuất Excel</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>38</v>
       </c>
       <c r="G11" s="17"/>
       <c r="H11" s="25" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct survey video task scope
The survey workflow only requires uploading an existing video. Rename the task, remove the direct-recording gap, and mark the delivered upload capability done.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4195,20 +4195,18 @@
       <c r="E44" s="39"/>
     </row>
     <row r="45">
-      <c r="A45" s="44" t="s">
-        <v>229</v>
+      <c r="A45" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Upload video khảo sát hiện trạng</t>
+        </is>
       </c>
       <c r="B45" s="37" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C45" s="37"/>
-      <c r="D45" s="44" t="inlineStr">
-        <is>
-          <t>Đã upload video; thiếu quay video trực tiếp trong ứng dụng.</t>
-        </is>
-      </c>
+      <c r="D45" s="48"/>
       <c r="E45" s="39"/>
     </row>
     <row r="46">

</xml_diff>

<commit_message>
Trace contract source leads via opportunities
Show converted source Leads on upstream Contracts through their source
Opportunity while enforcing Contract and Lead access independently.
Keep direct Contract creation and existing write contracts unchanged.

Add responsive links, conversion dates, loading and retry states, and
four-language guidance. Cover API scopes and real-stack navigation,
update the business guides, and mark the verified workbook task Done.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4315,13 +4315,13 @@
       </c>
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C54" s="37"/>
       <c r="D54" s="48" t="inlineStr">
         <is>
-          <t>Hợp đồng gắn Opportunity/Báo giá/Dự án; thiếu liên kết Lead trực tiếp.</t>
+          <t>Truy vết Lead qua Cơ hội nguồn theo quyền Lead; giữ liên kết Báo giá/Dự án.</t>
         </is>
       </c>
       <c r="E54" s="49"/>

</xml_diff>

<commit_message>
Add contract execution progress sources
Show separate work, effective QS and payment schedule measures.\nKeep Contract and source permissions independent with source links.\nSupport QS deep links and browser history without project drift.\nCover scope, history, recovery, localization and responsive flows.\nMark task 57 complete and document the approved business contract.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4358,13 +4358,13 @@
       </c>
       <c r="B57" s="37" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C57" s="37"/>
       <c r="D57" s="48" t="inlineStr">
         <is>
-          <t>Có lifecycle hợp đồng; thiếu tiến độ thực hiện từ công việc/nghiệm thu.</t>
+          <t>Tách công việc/QS/thanh toán gắn Hợp đồng; có nguồn đối chiếu, không gộp %.</t>
         </is>
       </c>
       <c r="E57" s="49"/>

</xml_diff>

<commit_message>
Refresh NICON workbook delivery progress
Reconcile current progress with source revision d884b3c6 and canonical
guides. Update contract care, revision comparison, QS/payment, CM and KPI
notes, and assess the outstanding demo requests.

Align status values and dropdowns with the repository delivery labels.
Preserve source requirements, estimates, formulas and workbook layout,
and document the assessment date without claiming deployment or UAT.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -3441,8 +3441,10 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú — đối chiếu source d884b3c6, 20/10/2026; không xác nhận host/UAT</t>
+        </is>
       </c>
       <c r="E1" s="2"/>
     </row>
@@ -3516,7 +3518,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C4" s="4"/>
@@ -3552,7 +3554,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C5" s="4"/>
@@ -3620,7 +3622,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C7" s="4"/>
@@ -3688,7 +3690,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C9" s="4"/>
@@ -3724,7 +3726,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C10" s="4"/>
@@ -3780,7 +3782,7 @@
       </c>
       <c r="B13" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C13" s="37"/>
@@ -3793,7 +3795,7 @@
       </c>
       <c r="B14" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C14" s="37"/>
@@ -3806,7 +3808,7 @@
       </c>
       <c r="B15" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C15" s="37"/>
@@ -3819,7 +3821,7 @@
       </c>
       <c r="B16" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C16" s="37"/>
@@ -3832,7 +3834,7 @@
       </c>
       <c r="B17" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C17" s="37"/>
@@ -3856,7 +3858,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C19" s="37"/>
@@ -3869,7 +3871,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C20" s="37"/>
@@ -3882,7 +3884,7 @@
       </c>
       <c r="B21" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C21" s="37"/>
@@ -3895,7 +3897,7 @@
       </c>
       <c r="B22" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C22" s="37"/>
@@ -3908,7 +3910,7 @@
       </c>
       <c r="B23" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C23" s="37"/>
@@ -3925,7 +3927,7 @@
       <c r="E24" s="39"/>
       <c r="J24" s="43" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3937,7 @@
       </c>
       <c r="B25" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C25" s="37"/>
@@ -3953,7 +3955,7 @@
       </c>
       <c r="B26" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C26" s="37"/>
@@ -3961,7 +3963,7 @@
       <c r="E26" s="39"/>
       <c r="J26" s="43" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3977,7 @@
       <c r="E27" s="39"/>
       <c r="J27" s="43" t="inlineStr">
         <is>
-          <t/>
+          <t xml:space="preserve">Open decision</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3987,7 @@
       </c>
       <c r="B28" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C28" s="37"/>
@@ -3998,7 +4000,7 @@
       </c>
       <c r="B29" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C29" s="37"/>
@@ -4011,7 +4013,7 @@
       </c>
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C30" s="37"/>
@@ -4024,7 +4026,7 @@
       </c>
       <c r="B31" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C31" s="37"/>
@@ -4039,7 +4041,7 @@
       </c>
       <c r="B32" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C32" s="37"/>
@@ -4052,7 +4054,7 @@
       </c>
       <c r="B33" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C33" s="37"/>
@@ -4074,7 +4076,7 @@
       </c>
       <c r="B35" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C35" s="37"/>
@@ -4087,7 +4089,7 @@
       </c>
       <c r="B36" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C36" s="37"/>
@@ -4100,7 +4102,7 @@
       </c>
       <c r="B37" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C37" s="37"/>
@@ -4113,7 +4115,7 @@
       </c>
       <c r="B38" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C38" s="37"/>
@@ -4126,7 +4128,7 @@
       </c>
       <c r="B39" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C39" s="37"/>
@@ -4139,7 +4141,7 @@
       </c>
       <c r="B40" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C40" s="37"/>
@@ -4152,7 +4154,7 @@
       </c>
       <c r="B41" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C41" s="37"/>
@@ -4174,7 +4176,7 @@
       </c>
       <c r="B43" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C43" s="37"/>
@@ -4187,7 +4189,7 @@
       </c>
       <c r="B44" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C44" s="37"/>
@@ -4202,7 +4204,7 @@
       </c>
       <c r="B45" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C45" s="37"/>
@@ -4215,7 +4217,7 @@
       </c>
       <c r="B46" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C46" s="37"/>
@@ -4228,7 +4230,7 @@
       </c>
       <c r="B47" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C47" s="37"/>
@@ -4241,7 +4243,7 @@
       </c>
       <c r="B48" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C48" s="37"/>
@@ -4254,7 +4256,7 @@
       </c>
       <c r="B49" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C49" s="37"/>
@@ -4267,7 +4269,7 @@
       </c>
       <c r="B50" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C50" s="37"/>
@@ -4280,7 +4282,7 @@
       </c>
       <c r="B51" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C51" s="37"/>
@@ -4302,7 +4304,7 @@
       </c>
       <c r="B53" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C53" s="37"/>
@@ -4315,7 +4317,7 @@
       </c>
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C54" s="37"/>
@@ -4332,7 +4334,7 @@
       </c>
       <c r="B55" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C55" s="37"/>
@@ -4345,7 +4347,7 @@
       </c>
       <c r="B56" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C56" s="37"/>
@@ -4358,7 +4360,7 @@
       </c>
       <c r="B57" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C57" s="37"/>
@@ -4375,7 +4377,7 @@
       </c>
       <c r="B58" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C58" s="37"/>
@@ -4388,7 +4390,7 @@
       </c>
       <c r="B59" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C59" s="37"/>
@@ -4401,7 +4403,7 @@
       </c>
       <c r="B60" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C60" s="37"/>
@@ -4431,13 +4433,13 @@
       </c>
       <c r="B62" s="37" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C62" s="37"/>
       <c r="D62" s="48" t="inlineStr">
         <is>
-          <t>Có lịch sử chăm sóc Khách hàng; thiếu timeline riêng theo Hợp đồng.</t>
+          <t xml:space="preserve">Timeline riêng theo HĐ; phân quyền, phân trang, retry; có lịch sử thì khóa đổi chiều.</t>
         </is>
       </c>
       <c r="E62" s="49"/>
@@ -4448,7 +4450,7 @@
       </c>
       <c r="B63" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C63" s="37"/>
@@ -4461,7 +4463,7 @@
       </c>
       <c r="B64" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C64" s="37"/>
@@ -4492,7 +4494,7 @@
       </c>
       <c r="B67" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C67" s="37"/>
@@ -4539,7 +4541,7 @@
       </c>
       <c r="B70" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C70" s="37"/>
@@ -4558,7 +4560,7 @@
       <c r="C71" s="37"/>
       <c r="D71" s="44" t="inlineStr">
         <is>
-          <t>Có quyết định/yêu cầu chỉnh sửa; thiếu thread phản hồi theo từng file của khách hàng.</t>
+          <t xml:space="preserve">Có bình luận nội bộ gắn từng file và ghi nhận ý kiến khách; chưa có thread/markup trực tiếp của khách.</t>
         </is>
       </c>
       <c r="E71" s="39"/>
@@ -4603,7 +4605,7 @@
       </c>
       <c r="B74" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C74" s="37"/>
@@ -4625,7 +4627,7 @@
       </c>
       <c r="B76" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C76" s="37"/>
@@ -4638,7 +4640,7 @@
       </c>
       <c r="B77" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C77" s="37"/>
@@ -4651,7 +4653,7 @@
       </c>
       <c r="B78" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C78" s="37"/>
@@ -4664,7 +4666,7 @@
       </c>
       <c r="B79" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C79" s="37"/>
@@ -4677,7 +4679,7 @@
       </c>
       <c r="B80" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C80" s="37"/>
@@ -4690,7 +4692,7 @@
       </c>
       <c r="B81" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C81" s="37"/>
@@ -4703,7 +4705,7 @@
       </c>
       <c r="B82" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C82" s="37"/>
@@ -4716,7 +4718,7 @@
       </c>
       <c r="B83" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C83" s="37"/>
@@ -4738,7 +4740,7 @@
       </c>
       <c r="B85" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C85" s="37"/>
@@ -4751,7 +4753,7 @@
       </c>
       <c r="B86" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C86" s="37"/>
@@ -4764,7 +4766,7 @@
       </c>
       <c r="B87" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C87" s="37"/>
@@ -4777,7 +4779,7 @@
       </c>
       <c r="B88" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C88" s="37"/>
@@ -4807,7 +4809,7 @@
       </c>
       <c r="B90" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C90" s="37"/>
@@ -4820,7 +4822,7 @@
       </c>
       <c r="B91" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C91" s="37"/>
@@ -4833,7 +4835,7 @@
       </c>
       <c r="B92" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C92" s="37"/>
@@ -4855,7 +4857,7 @@
       </c>
       <c r="B94" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C94" s="37"/>
@@ -4885,11 +4887,15 @@
       </c>
       <c r="B96" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="C96" s="37"/>
-      <c r="D96" s="44"/>
+      <c r="D96" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có so sánh metadata hai revision cùng bản vẽ; chưa so sánh nội dung/đồ họa của file.</t>
+        </is>
+      </c>
       <c r="E96" s="39"/>
     </row>
     <row r="97">
@@ -4898,7 +4904,7 @@
       </c>
       <c r="B97" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C97" s="37"/>
@@ -4911,7 +4917,7 @@
       </c>
       <c r="B98" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C98" s="37"/>
@@ -4924,7 +4930,7 @@
       </c>
       <c r="B99" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C99" s="37"/>
@@ -4937,11 +4943,15 @@
       </c>
       <c r="B100" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C100" s="37"/>
-      <c r="D100" s="44"/>
+      <c r="D100" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có lịch sử revision/IFC; chưa có luồng thông báo khi cập nhật revision cho các bộ phận.</t>
+        </is>
+      </c>
       <c r="E100" s="39"/>
     </row>
     <row r="101">
@@ -4959,7 +4969,7 @@
       </c>
       <c r="B102" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C102" s="37"/>
@@ -4989,7 +4999,7 @@
       </c>
       <c r="B104" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C104" s="37"/>
@@ -5002,7 +5012,7 @@
       </c>
       <c r="B105" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C105" s="37"/>
@@ -5015,7 +5025,7 @@
       </c>
       <c r="B106" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C106" s="37"/>
@@ -5028,7 +5038,7 @@
       </c>
       <c r="B107" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C107" s="37"/>
@@ -5041,7 +5051,7 @@
       </c>
       <c r="B108" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C108" s="37"/>
@@ -5072,7 +5082,7 @@
       </c>
       <c r="B111" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C111" s="37"/>
@@ -5085,7 +5095,7 @@
       </c>
       <c r="B112" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C112" s="37"/>
@@ -5104,7 +5114,7 @@
       <c r="C113" s="37"/>
       <c r="D113" s="80" t="inlineStr">
         <is>
-          <t>Có checklist theo dự án; thiếu template bắt buộc theo loại/quy mô công trình.</t>
+          <t xml:space="preserve">Có checklist theo Dự án; CM/NICON chưa duyệt template bắt buộc theo loại/quy mô công trình.</t>
         </is>
       </c>
       <c r="E113" s="81"/>
@@ -5115,7 +5125,7 @@
       </c>
       <c r="B114" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C114" s="37"/>
@@ -5128,7 +5138,7 @@
       </c>
       <c r="B115" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C115" s="37"/>
@@ -5141,7 +5151,7 @@
       </c>
       <c r="B116" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C116" s="37"/>
@@ -5154,7 +5164,7 @@
       </c>
       <c r="B117" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C117" s="37"/>
@@ -5167,7 +5177,7 @@
       </c>
       <c r="B118" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C118" s="37"/>
@@ -5189,7 +5199,7 @@
       </c>
       <c r="B120" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C120" s="37"/>
@@ -5202,7 +5212,7 @@
       </c>
       <c r="B121" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C121" s="37"/>
@@ -5215,7 +5225,7 @@
       </c>
       <c r="B122" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C122" s="37"/>
@@ -5228,7 +5238,7 @@
       </c>
       <c r="B123" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C123" s="37"/>
@@ -5241,7 +5251,7 @@
       </c>
       <c r="B124" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C124" s="37"/>
@@ -5254,7 +5264,7 @@
       </c>
       <c r="B125" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C125" s="37"/>
@@ -5267,7 +5277,7 @@
       </c>
       <c r="B126" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C126" s="37"/>
@@ -5280,7 +5290,7 @@
       </c>
       <c r="B127" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C127" s="37"/>
@@ -5345,7 +5355,7 @@
       </c>
       <c r="B132" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C132" s="37"/>
@@ -5358,7 +5368,7 @@
       </c>
       <c r="B133" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C133" s="37"/>
@@ -5371,7 +5381,7 @@
       </c>
       <c r="B134" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C134" s="37"/>
@@ -5384,7 +5394,7 @@
       </c>
       <c r="B135" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C135" s="37"/>
@@ -5431,7 +5441,7 @@
       </c>
       <c r="B138" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C138" s="37"/>
@@ -5453,7 +5463,7 @@
       </c>
       <c r="B140" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C140" s="37"/>
@@ -5466,7 +5476,7 @@
       </c>
       <c r="B141" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C141" s="37"/>
@@ -5513,7 +5523,7 @@
       </c>
       <c r="B144" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C144" s="37"/>
@@ -5526,7 +5536,7 @@
       </c>
       <c r="B145" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C145" s="37"/>
@@ -5539,7 +5549,7 @@
       </c>
       <c r="B146" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C146" s="37"/>
@@ -5552,7 +5562,7 @@
       </c>
       <c r="B147" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C147" s="37"/>
@@ -5565,7 +5575,7 @@
       </c>
       <c r="B148" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C148" s="37"/>
@@ -5578,7 +5588,7 @@
       </c>
       <c r="B149" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C149" s="37"/>
@@ -5600,7 +5610,7 @@
       </c>
       <c r="B151" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C151" s="37"/>
@@ -5613,7 +5623,7 @@
       </c>
       <c r="B152" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C152" s="37"/>
@@ -5632,7 +5642,7 @@
       <c r="C153" s="37"/>
       <c r="D153" s="99" t="inlineStr">
         <is>
-          <t>Có dữ liệu QA/QC; thiếu checklist nghiệm thu bắt buộc theo template NICON.</t>
+          <t xml:space="preserve">Có template engine QA/QC; còn chờ CM duyệt mapping/checklist ISO NICON để publish mẫu sản xuất.</t>
         </is>
       </c>
       <c r="E153" s="86"/>
@@ -5643,7 +5653,7 @@
       </c>
       <c r="B154" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C154" s="37"/>
@@ -5656,7 +5666,7 @@
       </c>
       <c r="B155" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C155" s="37"/>
@@ -5686,7 +5696,7 @@
       </c>
       <c r="B157" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C157" s="37"/>
@@ -5699,7 +5709,7 @@
       </c>
       <c r="B158" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C158" s="37"/>
@@ -5712,7 +5722,7 @@
       </c>
       <c r="B159" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C159" s="37"/>
@@ -5785,7 +5795,7 @@
       </c>
       <c r="B164" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C164" s="37"/>
@@ -5815,7 +5825,7 @@
       </c>
       <c r="B166" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C166" s="37"/>
@@ -5828,7 +5838,7 @@
       </c>
       <c r="B167" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C167" s="37"/>
@@ -5841,7 +5851,7 @@
       </c>
       <c r="B168" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C168" s="37"/>
@@ -5863,7 +5873,7 @@
       </c>
       <c r="B170" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C170" s="37"/>
@@ -5893,7 +5903,7 @@
       </c>
       <c r="B172" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C172" s="37"/>
@@ -5906,7 +5916,7 @@
       </c>
       <c r="B173" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C173" s="37"/>
@@ -5936,7 +5946,7 @@
       </c>
       <c r="B175" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C175" s="37"/>
@@ -5949,7 +5959,7 @@
       </c>
       <c r="B176" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C176" s="37"/>
@@ -5971,7 +5981,7 @@
       </c>
       <c r="B178" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C178" s="37"/>
@@ -5984,7 +5994,7 @@
       </c>
       <c r="B179" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C179" s="37"/>
@@ -6014,7 +6024,7 @@
       </c>
       <c r="B181" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C181" s="37"/>
@@ -6027,7 +6037,7 @@
       </c>
       <c r="B182" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C182" s="37"/>
@@ -6040,7 +6050,7 @@
       </c>
       <c r="B183" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C183" s="37"/>
@@ -6053,7 +6063,7 @@
       </c>
       <c r="B184" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C184" s="37"/>
@@ -6066,7 +6076,7 @@
       </c>
       <c r="B185" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C185" s="37"/>
@@ -6079,7 +6089,7 @@
       </c>
       <c r="B186" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C186" s="37"/>
@@ -6110,7 +6120,7 @@
       </c>
       <c r="B189" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C189" s="37"/>
@@ -6123,7 +6133,7 @@
       </c>
       <c r="B190" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C190" s="37"/>
@@ -6136,7 +6146,7 @@
       </c>
       <c r="B191" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C191" s="37"/>
@@ -6149,7 +6159,7 @@
       </c>
       <c r="B192" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C192" s="37"/>
@@ -6179,7 +6189,7 @@
       </c>
       <c r="B194" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C194" s="37"/>
@@ -6192,7 +6202,7 @@
       </c>
       <c r="B195" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C195" s="37"/>
@@ -6231,7 +6241,7 @@
       </c>
       <c r="B198" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C198" s="37"/>
@@ -6244,7 +6254,7 @@
       </c>
       <c r="B199" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C199" s="37"/>
@@ -6257,7 +6267,7 @@
       </c>
       <c r="B200" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C200" s="37"/>
@@ -6270,7 +6280,7 @@
       </c>
       <c r="B201" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C201" s="37"/>
@@ -6283,7 +6293,7 @@
       </c>
       <c r="B202" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C202" s="37"/>
@@ -6296,7 +6306,7 @@
       </c>
       <c r="B203" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C203" s="37"/>
@@ -6309,7 +6319,7 @@
       </c>
       <c r="B204" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C204" s="37"/>
@@ -6348,7 +6358,7 @@
       </c>
       <c r="B207" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C207" s="37"/>
@@ -6361,7 +6371,7 @@
       </c>
       <c r="B208" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C208" s="37"/>
@@ -6374,7 +6384,7 @@
       </c>
       <c r="B209" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C209" s="37"/>
@@ -6387,7 +6397,7 @@
       </c>
       <c r="B210" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C210" s="37"/>
@@ -6400,7 +6410,7 @@
       </c>
       <c r="B211" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C211" s="37"/>
@@ -6456,7 +6466,7 @@
       </c>
       <c r="B215" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C215" s="37"/>
@@ -6469,7 +6479,7 @@
       </c>
       <c r="B216" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C216" s="37"/>
@@ -6499,7 +6509,7 @@
       </c>
       <c r="B218" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C218" s="37"/>
@@ -6512,7 +6522,7 @@
       </c>
       <c r="B219" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C219" s="37"/>
@@ -6551,7 +6561,7 @@
       </c>
       <c r="B222" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C222" s="37"/>
@@ -6564,7 +6574,7 @@
       </c>
       <c r="B223" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C223" s="37"/>
@@ -6577,7 +6587,7 @@
       </c>
       <c r="B224" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C224" s="37"/>
@@ -6590,7 +6600,7 @@
       </c>
       <c r="B225" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C225" s="37"/>
@@ -6603,7 +6613,7 @@
       </c>
       <c r="B226" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C226" s="37"/>
@@ -6616,7 +6626,7 @@
       </c>
       <c r="B227" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C227" s="37"/>
@@ -6672,7 +6682,7 @@
       </c>
       <c r="B231" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C231" s="37"/>
@@ -6685,7 +6695,7 @@
       </c>
       <c r="B232" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C232" s="37"/>
@@ -6698,7 +6708,7 @@
       </c>
       <c r="B233" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C233" s="37"/>
@@ -6728,7 +6738,7 @@
       </c>
       <c r="B235" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C235" s="37"/>
@@ -6750,7 +6760,7 @@
       </c>
       <c r="B237" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C237" s="37"/>
@@ -6763,7 +6773,7 @@
       </c>
       <c r="B238" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C238" s="37"/>
@@ -6793,7 +6803,7 @@
       </c>
       <c r="B240" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C240" s="37"/>
@@ -6806,7 +6816,7 @@
       </c>
       <c r="B241" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C241" s="37"/>
@@ -6819,7 +6829,7 @@
       </c>
       <c r="B242" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C242" s="37"/>
@@ -6850,7 +6860,7 @@
       </c>
       <c r="B245" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C245" s="37"/>
@@ -6863,7 +6873,7 @@
       </c>
       <c r="B246" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C246" s="37"/>
@@ -6876,7 +6886,7 @@
       </c>
       <c r="B247" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C247" s="37"/>
@@ -6895,7 +6905,7 @@
       <c r="C248" s="37"/>
       <c r="D248" s="30" t="inlineStr">
         <is>
-          <t>Có mốc thanh toán; thiếu gate theo nghiệm thu/QS được duyệt.</t>
+          <t xml:space="preserve">Có mốc phải thu và tham chiếu QS Upstream; chưa có dossier/gate thu tiền theo ISO đã duyệt.</t>
         </is>
       </c>
       <c r="E248" s="101"/>
@@ -6923,7 +6933,7 @@
       </c>
       <c r="B250" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C250" s="37"/>
@@ -6936,7 +6946,7 @@
       </c>
       <c r="B251" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C251" s="37"/>
@@ -6949,7 +6959,7 @@
       </c>
       <c r="B252" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C252" s="37"/>
@@ -6962,7 +6972,7 @@
       </c>
       <c r="B253" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C253" s="37"/>
@@ -6984,7 +6994,7 @@
       </c>
       <c r="B255" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C255" s="37"/>
@@ -6997,7 +7007,7 @@
       </c>
       <c r="B256" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C256" s="37"/>
@@ -7010,7 +7020,7 @@
       </c>
       <c r="B257" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C257" s="37"/>
@@ -7029,7 +7039,7 @@
       <c r="C258" s="37"/>
       <c r="D258" s="30" t="inlineStr">
         <is>
-          <t>Có mốc thanh toán Downstream; thiếu liên kết tiến độ/QS đủ điều kiện.</t>
+          <t xml:space="preserve">Có mốc Downstream và QS liên kết Payment Request; chưa có gate ISO cho từng loại gói.</t>
         </is>
       </c>
       <c r="E258" s="101"/>
@@ -7040,7 +7050,7 @@
       </c>
       <c r="B259" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C259" s="37"/>
@@ -7059,7 +7069,7 @@
       <c r="C260" s="37"/>
       <c r="D260" s="30" t="inlineStr">
         <is>
-          <t>Có lifecycle hợp đồng; thiếu tiến độ thi công thực tế theo gói thầu.</t>
+          <t xml:space="preserve">Có nguồn công việc, QS và mốc thanh toán theo HĐ; chưa có % tiến độ gói thầu theo baseline.</t>
         </is>
       </c>
       <c r="E260" s="101"/>
@@ -7076,7 +7086,7 @@
       <c r="C261" s="37"/>
       <c r="D261" s="30" t="inlineStr">
         <is>
-          <t>Có Payment Request/Paid; thiếu lịch sử chi tiền có chứng từ đối soát.</t>
+          <t xml:space="preserve">Có Payment Request/Paid, lịch sử revision và sửa hồ sơ khi QS bị thay thế; thiếu sổ chi đối soát.</t>
         </is>
       </c>
       <c r="E261" s="101"/>
@@ -7087,7 +7097,7 @@
       </c>
       <c r="B262" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C262" s="37"/>
@@ -7109,7 +7119,7 @@
       </c>
       <c r="B264" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C264" s="37"/>
@@ -7139,7 +7149,7 @@
       </c>
       <c r="B266" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C266" s="37"/>
@@ -7158,7 +7168,7 @@
       <c r="C267" s="37"/>
       <c r="D267" s="30" t="inlineStr">
         <is>
-          <t>VO hiện gắn Hợp đồng Upstream; thiếu VO cho Hợp đồng Downstream.</t>
+          <t xml:space="preserve">API/UI VO dùng chung theo HĐ; chưa có test riêng xác nhận đầy đủ luồng VO Downstream.</t>
         </is>
       </c>
       <c r="E267" s="101"/>
@@ -7169,7 +7179,7 @@
       </c>
       <c r="B268" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C268" s="37"/>
@@ -7182,7 +7192,7 @@
       </c>
       <c r="B269" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C269" s="37"/>
@@ -7195,7 +7205,7 @@
       </c>
       <c r="B270" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C270" s="37"/>
@@ -7208,7 +7218,7 @@
       </c>
       <c r="B271" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C271" s="37"/>
@@ -7264,7 +7274,7 @@
       </c>
       <c r="B275" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C275" s="37"/>
@@ -7311,7 +7321,7 @@
       </c>
       <c r="B278" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C278" s="37"/>
@@ -7324,7 +7334,7 @@
       </c>
       <c r="B279" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C279" s="37"/>
@@ -7346,7 +7356,7 @@
       </c>
       <c r="B281" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C281" s="37"/>
@@ -7359,7 +7369,7 @@
       </c>
       <c r="B282" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C282" s="37"/>
@@ -7372,7 +7382,7 @@
       </c>
       <c r="B283" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C283" s="37"/>
@@ -7385,11 +7395,15 @@
       </c>
       <c r="B284" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C284" s="37"/>
-      <c r="D284" s="30"/>
+      <c r="D284" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CM có giá trị QS được duyệt/kỳ nghiệm thu; chưa có nguồn chi phí thực tế và công thức so với dự toán.</t>
+        </is>
+      </c>
       <c r="E284" s="101"/>
     </row>
     <row r="285">
@@ -7398,7 +7412,7 @@
       </c>
       <c r="B285" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C285" s="37"/>
@@ -7411,7 +7425,7 @@
       </c>
       <c r="B286" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C286" s="37"/>
@@ -7424,7 +7438,7 @@
       </c>
       <c r="B287" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C287" s="37"/>
@@ -7455,7 +7469,7 @@
       </c>
       <c r="B290" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C290" s="37"/>
@@ -7485,7 +7499,7 @@
       </c>
       <c r="B292" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C292" s="37"/>
@@ -7498,7 +7512,7 @@
       </c>
       <c r="B293" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C293" s="37"/>
@@ -7545,7 +7559,7 @@
       </c>
       <c r="B296" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C296" s="37"/>
@@ -7558,7 +7572,7 @@
       </c>
       <c r="B297" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C297" s="37"/>
@@ -7580,7 +7594,7 @@
       </c>
       <c r="B299" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C299" s="37"/>
@@ -7593,7 +7607,7 @@
       </c>
       <c r="B300" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C300" s="37"/>
@@ -7606,7 +7620,7 @@
       </c>
       <c r="B301" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C301" s="37"/>
@@ -7619,7 +7633,7 @@
       </c>
       <c r="B302" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C302" s="37"/>
@@ -7632,7 +7646,7 @@
       </c>
       <c r="B303" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C303" s="37"/>
@@ -7645,7 +7659,7 @@
       </c>
       <c r="B304" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C304" s="37"/>
@@ -7658,7 +7672,7 @@
       </c>
       <c r="B305" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C305" s="37"/>
@@ -7671,7 +7685,7 @@
       </c>
       <c r="B306" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C306" s="37"/>
@@ -7684,7 +7698,7 @@
       </c>
       <c r="B307" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C307" s="37"/>
@@ -7721,7 +7735,7 @@
       <c r="C310" s="37"/>
       <c r="D310" s="85" t="inlineStr">
         <is>
-          <t>Có tiến độ thiết kế và đếm task thi công; thiếu % thi công theo baseline.</t>
+          <t xml:space="preserve">Có task/Gantt và CM theo trạng thái hiện tại; chưa có % thi công theo baseline đã công bố.</t>
         </is>
       </c>
       <c r="E310" s="86"/>
@@ -7749,7 +7763,7 @@
       </c>
       <c r="B312" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C312" s="37"/>
@@ -7779,7 +7793,7 @@
       </c>
       <c r="B314" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C314" s="37"/>
@@ -7792,7 +7806,7 @@
       </c>
       <c r="B315" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C315" s="37"/>
@@ -7805,7 +7819,7 @@
       </c>
       <c r="B316" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C316" s="37"/>
@@ -7833,7 +7847,7 @@
       <c r="C318" s="37"/>
       <c r="D318" s="85" t="inlineStr">
         <is>
-          <t>Có số lượng nghiệm thu; thiếu tỷ lệ đạt/không đạt có mẫu số chuẩn.</t>
+          <t xml:space="preserve">Có đếm nghiệm thu/QS riêng hai chiều; số hồ sơ không phải tỷ lệ hay khối lượng vật lý hoàn thành.</t>
         </is>
       </c>
       <c r="E318" s="86"/>
@@ -7844,7 +7858,7 @@
       </c>
       <c r="B319" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C319" s="37"/>
@@ -7857,7 +7871,7 @@
       </c>
       <c r="B320" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C320" s="37"/>
@@ -7876,7 +7890,7 @@
       <c r="C321" s="37"/>
       <c r="D321" s="97" t="inlineStr">
         <is>
-          <t>Có file nghiệm thu theo hồ sơ; thiếu danh mục tổng hợp biên bản theo Dự án.</t>
+          <t xml:space="preserve">CM có nguồn QA/QC và link đối chiếu; chưa tự tập hợp đầy đủ biên bản nghiệm thu của Dự án.</t>
         </is>
       </c>
       <c r="E321" s="98"/>
@@ -7947,7 +7961,7 @@
       </c>
       <c r="B326" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C326" s="37"/>
@@ -7960,11 +7974,15 @@
       </c>
       <c r="B327" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="C327" s="37"/>
-      <c r="D327" s="85"/>
+      <c r="D327" s="85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có lịch mốc phải thu, ngày xác nhận thu và quá hạn; chưa có sổ phải thu đối soát chứng từ.</t>
+        </is>
+      </c>
       <c r="E327" s="86"/>
     </row>
     <row r="328">
@@ -7973,7 +7991,7 @@
       </c>
       <c r="B328" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C328" s="37"/>
@@ -7986,7 +8004,7 @@
       </c>
       <c r="B329" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C329" s="37"/>
@@ -7999,7 +8017,7 @@
       </c>
       <c r="B330" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C330" s="37"/>
@@ -8012,7 +8030,7 @@
       </c>
       <c r="B331" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C331" s="37"/>
@@ -8025,11 +8043,15 @@
       </c>
       <c r="B332" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="C332" s="37"/>
-      <c r="D332" s="85"/>
+      <c r="D332" s="85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có xuất báo cáo giá trị HĐ/mốc thanh toán; chưa xuất sổ thu–chi/P&amp;L thực tế.</t>
+        </is>
+      </c>
       <c r="E332" s="86"/>
     </row>
     <row r="333">
@@ -8081,7 +8103,7 @@
       </c>
       <c r="B336" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C336" s="37"/>
@@ -8094,7 +8116,7 @@
       </c>
       <c r="B337" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C337" s="37"/>
@@ -8107,7 +8129,7 @@
       </c>
       <c r="B338" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C338" s="37"/>
@@ -8163,7 +8185,7 @@
       </c>
       <c r="B342" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C342" s="37"/>
@@ -8176,7 +8198,7 @@
       </c>
       <c r="B343" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C343" s="37"/>
@@ -8189,7 +8211,7 @@
       </c>
       <c r="B344" s="37" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
       <c r="C344" s="37"/>
@@ -8202,7 +8224,7 @@
       </c>
       <c r="B345" s="37" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C345" s="37"/>
@@ -8255,7 +8277,7 @@
       <c r="C348" s="37"/>
       <c r="D348" s="85" t="inlineStr">
         <is>
-          <t>Có dashboard vận hành; thiếu tổng hợp cảnh báo liên module và drill-down nguồn.</t>
+          <t xml:space="preserve">Có dashboard và CM: QS hai chiều, giá trị/kỳ, QA/QC, HSE; còn thiếu tài chính thực tế và S-Curve.</t>
         </is>
       </c>
       <c r="E348" s="86"/>
@@ -11015,7 +11037,7 @@
   </mergeCells>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B4:B5 B7 B9:B10 B13:B17 B19:B23 B25:B26 B28:B41 B43:B51 B53:B64 B67:B74 B76:B83 B85:B92 B94:B100 B102:B108 B111:B118 B120:B127 B130:B138 B140:B149 B151:B159 B161:C168 B170:C176 B178:C186 B189:C195 B197:C204 B206:C212 B214:C219 B221:C227 B229:C235 B237:C242 B245:C253 B255:C262 B264:C271 B273:C279 B281:C287 B290:C297 B299:C307 B310:C316 B318:C324 B326:C332 B334:C340 B342:C348">
-      <formula1>Nicon!$J$24:$J$26</formula1>
+      <formula1>Nicon!$J$24:$J$27</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
@@ -11343,127 +11365,211 @@
       <c r="A2" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="21"/>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="21"/>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="21"/>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="21"/>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="21"/>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="21"/>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="21"/>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="21"/>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="21"/>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="21"/>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="21"/>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="21"/>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="21"/>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B15" s="21"/>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="21"/>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B17" s="21"/>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="21"/>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="B19" s="21"/>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="B20" s="21"/>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B21" s="21"/>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B22" s="21"/>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -11506,8 +11612,10 @@
       <c r="E1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="11" t="s">
-        <v>10</v>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghi chú — đối chiếu source d884b3c6, 20/10/2026</t>
+        </is>
       </c>
       <c r="G1" s="12" t="s">
         <v>12</v>
@@ -11538,7 +11646,7 @@
       <c r="G2" s="17"/>
       <c r="H2" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11560,7 +11668,7 @@
       <c r="G3" s="17"/>
       <c r="H3" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11582,7 +11690,7 @@
       <c r="G4" s="17"/>
       <c r="H4" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11606,7 +11714,7 @@
       <c r="G5" s="17"/>
       <c r="H5" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11628,7 +11736,7 @@
       <c r="G6" s="17"/>
       <c r="H6" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11650,7 +11758,7 @@
       <c r="G7" s="17"/>
       <c r="H7" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11672,7 +11780,7 @@
       <c r="G8" s="17"/>
       <c r="H8" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11696,7 +11804,7 @@
       <c r="G9" s="17"/>
       <c r="H9" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11718,7 +11826,7 @@
       <c r="G10" s="17"/>
       <c r="H10" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11742,7 +11850,7 @@
       <c r="G11" s="17"/>
       <c r="H11" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11766,7 +11874,7 @@
       <c r="G12" s="17"/>
       <c r="H12" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11788,7 +11896,7 @@
       <c r="G13" s="17"/>
       <c r="H13" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11810,7 +11918,7 @@
       <c r="G14" s="17"/>
       <c r="H14" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11832,7 +11940,7 @@
       <c r="G15" s="17"/>
       <c r="H15" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11856,7 +11964,7 @@
       <c r="G16" s="17"/>
       <c r="H16" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11878,7 +11986,7 @@
       <c r="G17" s="17"/>
       <c r="H17" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11900,7 +12008,7 @@
       <c r="G18" s="17"/>
       <c r="H18" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11924,7 +12032,7 @@
       <c r="G19" s="17"/>
       <c r="H19" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11946,7 +12054,7 @@
       <c r="G20" s="17"/>
       <c r="H20" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11962,13 +12070,15 @@
       <c r="E21" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="F21" s="17" t="s">
-        <v>38</v>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có tiến độ theo HĐ, nguồn Lead và timeline chăm sóc riêng; có lịch sử thì khóa đổi chiều.</t>
+        </is>
       </c>
       <c r="G21" s="17"/>
       <c r="H21" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -11994,7 +12104,7 @@
       <c r="G22" s="17"/>
       <c r="H22" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12016,7 +12126,7 @@
       <c r="G23" s="17"/>
       <c r="H23" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12148,7 @@
       <c r="G24" s="17"/>
       <c r="H24" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12062,7 +12172,7 @@
       <c r="G25" s="17"/>
       <c r="H25" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12084,7 +12194,7 @@
       <c r="G26" s="17"/>
       <c r="H26" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12102,7 +12212,7 @@
       </c>
       <c r="F27" s="103" t="inlineStr">
         <is>
-          <t>Detail page | Thiếu trình duyệt/ký trực tiếp trên portal khách hàng và markup từng file.</t>
+          <t xml:space="preserve">Có review nội bộ gắn file và ghi nhận quyết định khách; chưa có portal ký/markup trực tiếp.</t>
         </is>
       </c>
       <c r="G27" s="17"/>
@@ -12132,7 +12242,7 @@
       <c r="G28" s="17"/>
       <c r="H28" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12154,7 +12264,7 @@
       <c r="G29" s="17"/>
       <c r="H29" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12176,7 +12286,7 @@
       <c r="G30" s="17"/>
       <c r="H30" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12200,7 +12310,7 @@
       <c r="G31" s="17"/>
       <c r="H31" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12222,7 +12332,7 @@
       <c r="G32" s="17"/>
       <c r="H32" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12240,7 +12350,7 @@
       </c>
       <c r="F33" s="103" t="inlineStr">
         <is>
-          <t>Detail page | Thiếu markup/review chéo trực tiếp trên từng file bản vẽ.</t>
+          <t xml:space="preserve">Có review nội bộ gắn file; chưa có markup đồ họa trực tiếp trên từng bản vẽ.</t>
         </is>
       </c>
       <c r="G33" s="17"/>
@@ -12270,7 +12380,7 @@
       <c r="G34" s="17"/>
       <c r="H34" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12286,13 +12396,15 @@
       <c r="E35" s="23" t="s">
         <v>195</v>
       </c>
-      <c r="F35" s="17" t="s">
-        <v>33</v>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có tạo revision kèm lý do/ghi chú; chưa có sửa revision đã ghi nhận.</t>
+        </is>
       </c>
       <c r="G35" s="17"/>
       <c r="H35" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
     </row>
@@ -12308,13 +12420,15 @@
       <c r="E36" s="23" t="s">
         <v>202</v>
       </c>
-      <c r="F36" s="17" t="s">
-        <v>38</v>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có lịch sử và so sánh metadata revision; chưa có diff nội dung file.</t>
+        </is>
       </c>
       <c r="G36" s="17"/>
       <c r="H36" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12338,7 +12452,7 @@
       <c r="G37" s="17"/>
       <c r="H37" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12360,7 +12474,7 @@
       <c r="G38" s="17"/>
       <c r="H38" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12410,7 +12524,7 @@
       <c r="G40" s="17"/>
       <c r="H40" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12432,7 +12546,7 @@
       <c r="G41" s="17"/>
       <c r="H41" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12454,7 +12568,7 @@
       <c r="G42" s="17"/>
       <c r="H42" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12480,7 +12594,7 @@
       <c r="G43" s="17"/>
       <c r="H43" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12502,7 +12616,7 @@
       <c r="G44" s="17"/>
       <c r="H44" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12520,7 +12634,7 @@
       </c>
       <c r="F45" s="103" t="inlineStr">
         <is>
-          <t>Detail page + Gantt UI | Thiếu baseline WBS/S-Curve, critical path và cảnh báo lệch &gt;5%.</t>
+          <t xml:space="preserve">Có task/Gantt và readiness gate; thiếu baseline WBS/S-Curve có cấu trúc, critical path và lệch &gt;5%.</t>
         </is>
       </c>
       <c r="G45" s="17"/>
@@ -12550,7 +12664,7 @@
       <c r="G46" s="17"/>
       <c r="H46" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12572,7 +12686,7 @@
       <c r="G47" s="17"/>
       <c r="H47" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12620,7 +12734,7 @@
       <c r="G49" s="17"/>
       <c r="H49" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12642,7 +12756,7 @@
       <c r="G50" s="17"/>
       <c r="H50" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12660,7 +12774,7 @@
       </c>
       <c r="F51" s="103" t="inlineStr">
         <is>
-          <t>Detail page | Thiếu checklist nghiệm thu NICON và kết quả Đạt/Không đạt riêng.</t>
+          <t xml:space="preserve">Có QA/QC template engine, IFC/evidence; chờ CM duyệt mapping ISO, chưa đủ gate nghiệm thu mục tiêu.</t>
         </is>
       </c>
       <c r="G51" s="17"/>
@@ -12690,7 +12804,7 @@
       <c r="G52" s="17"/>
       <c r="H52" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12712,7 +12826,7 @@
       <c r="G53" s="17"/>
       <c r="H53" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12760,7 +12874,7 @@
       <c r="G55" s="17"/>
       <c r="H55" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12782,7 +12896,7 @@
       <c r="G56" s="17"/>
       <c r="H56" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12830,7 +12944,7 @@
       <c r="G58" s="17"/>
       <c r="H58" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12852,7 +12966,7 @@
       <c r="G59" s="17"/>
       <c r="H59" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12902,7 +13016,7 @@
       <c r="G61" s="17"/>
       <c r="H61" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12924,7 +13038,7 @@
       <c r="G62" s="17"/>
       <c r="H62" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12946,7 +13060,7 @@
       <c r="G63" s="17"/>
       <c r="H63" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12970,7 +13084,7 @@
       <c r="G64" s="17"/>
       <c r="H64" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -12992,7 +13106,7 @@
       <c r="G65" s="17"/>
       <c r="H65" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13014,7 +13128,7 @@
       <c r="G66" s="17"/>
       <c r="H66" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13038,7 +13152,7 @@
       <c r="G67" s="17"/>
       <c r="H67" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13084,7 +13198,7 @@
       <c r="G69" s="17"/>
       <c r="H69" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13108,7 +13222,7 @@
       <c r="G70" s="17"/>
       <c r="H70" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13130,7 +13244,7 @@
       <c r="G71" s="17"/>
       <c r="H71" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13152,7 +13266,7 @@
       <c r="G72" s="17"/>
       <c r="H72" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13176,7 +13290,7 @@
       <c r="G73" s="17"/>
       <c r="H73" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13198,7 +13312,7 @@
       <c r="G74" s="17"/>
       <c r="H74" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13246,7 +13360,7 @@
       <c r="G76" s="17"/>
       <c r="H76" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13272,7 +13386,7 @@
       <c r="G77" s="17"/>
       <c r="H77" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13294,7 +13408,7 @@
       <c r="G78" s="17"/>
       <c r="H78" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13312,7 +13426,7 @@
       </c>
       <c r="F79" s="103" t="inlineStr">
         <is>
-          <t>Detail page | Có Hợp đồng/mốc/VO; thiếu sổ phải thu và thu tiền đối soát chứng từ.</t>
+          <t xml:space="preserve">Có HĐ, mốc, ngày thu và VO; thiếu sổ phải thu đối soát chứng từ.</t>
         </is>
       </c>
       <c r="G79" s="17"/>
@@ -13342,7 +13456,7 @@
       <c r="G80" s="17"/>
       <c r="H80" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13478,7 @@
       <c r="G81" s="17"/>
       <c r="H81" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13382,7 +13496,7 @@
       </c>
       <c r="F82" s="103" t="inlineStr">
         <is>
-          <t>Detail page | Có Hợp đồng/mốc/Payment Request; thiếu sổ phải trả và dossier thanh toán.</t>
+          <t xml:space="preserve">Có Payment Request gắn QS Downstream, revision khôi phục; thiếu sổ phải trả và dossier ISO ba section.</t>
         </is>
       </c>
       <c r="G82" s="17"/>
@@ -13412,7 +13526,7 @@
       <c r="G83" s="17"/>
       <c r="H83" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13434,7 +13548,7 @@
       <c r="G84" s="17"/>
       <c r="H84" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13456,7 +13570,7 @@
       <c r="G85" s="17"/>
       <c r="H85" s="25" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -13480,7 +13594,7 @@
       <c r="G86" s="17"/>
       <c r="H86" s="25" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
     </row>
@@ -13504,7 +13618,7 @@
       <c r="G87" s="17"/>
       <c r="H87" s="25" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
     </row>
@@ -13580,7 +13694,7 @@
       </c>
       <c r="F90" s="103" t="inlineStr">
         <is>
-          <t>Dashboard | Có dashboard vận hành; thiếu tài chính thực tế, tồn kho và KPI đủ 11 vị trí.</t>
+          <t xml:space="preserve">Có dashboard vận hành và CM: QS hai chiều, giá trị/kỳ, QA/QC, HSE; thiếu ledger, S-Curve, đủ 11 vị trí.</t>
         </is>
       </c>
       <c r="G90" s="17"/>
@@ -13606,7 +13720,7 @@
       </c>
       <c r="F91" s="103" t="inlineStr">
         <is>
-          <t>Report | Có báo cáo Dự án; thiếu số liệu tài chính, BOQ usage và vendor performance.</t>
+          <t xml:space="preserve">Có báo cáo Dự án, nguồn CM và export; thiếu tài chính thực tế, BOQ usage và vendor performance.</t>
         </is>
       </c>
       <c r="G91" s="17"/>
@@ -13736,7 +13850,7 @@
       </c>
       <c r="F96" s="103" t="inlineStr">
         <is>
-          <t>Report + Export | Có export KPI hiện tại; thiếu Google Sheets/PDF theo toàn bộ vị trí.</t>
+          <t xml:space="preserve">Có CSV KPI theo nhân viên/kỳ; chưa có Google Sheets/PDF và lưu tự động lên Drive.</t>
         </is>
       </c>
       <c r="G96" s="79">
@@ -13762,7 +13876,7 @@
       </c>
       <c r="F97" s="103" t="inlineStr">
         <is>
-          <t>Workflow/admin | Có khóa kỳ/snapshot; thiếu phạm vi HR/Admin theo framework NICON.</t>
+          <t xml:space="preserve">Có khóa kỳ/snapshot và quyền manage; role HR mặc định chưa có quyền KPI.</t>
         </is>
       </c>
       <c r="G97" s="79">
@@ -13788,7 +13902,7 @@
       </c>
       <c r="F98" s="103" t="inlineStr">
         <is>
-          <t>Notification/audit | Có audit KPI/export; thiếu cảnh báo điểm bất thường theo rule đã duyệt.</t>
+          <t xml:space="preserve">Có audit/export và cảnh báo điểm thấp theo ngưỡng; chưa phủ rule/cảnh báo đủ 11 vị trí.</t>
         </is>
       </c>
       <c r="G98" s="79">
@@ -13906,7 +14020,7 @@
       <c r="G102" s="17"/>
       <c r="H102" s="25" t="inlineStr">
         <is>
-          <t>Not Implement</t>
+          <t xml:space="preserve">Target</t>
         </is>
       </c>
     </row>
@@ -13988,7 +14102,7 @@
       <c r="G105" s="93"/>
       <c r="H105" s="89" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -14014,7 +14128,7 @@
       <c r="G106" s="93"/>
       <c r="H106" s="89" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -14040,7 +14154,7 @@
       <c r="G107" s="93"/>
       <c r="H107" s="89" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -14066,7 +14180,7 @@
       <c r="G108" s="93"/>
       <c r="H108" s="89" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
     </row>
@@ -17921,7 +18035,7 @@
   </mergeCells>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H2:H108">
-      <formula1>"Done,Partial,Not Implement"</formula1>
+      <formula1>"Implemented,Partial,Target,Open decision"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Add automatic contract reminder emails
Schedule customer renewal and end-date emails per contract after
reviewing the rendered message. Manage both templates in admin
settings, validate recipient scope and preserve approved snapshots.

Persist delivery claims and history, expose uncertain SMTP outcomes,
and block deletion while a message is sending. Add focused unit,
integration and browser coverage, and update NICON guides and progress.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4416,13 +4416,13 @@
       </c>
       <c r="B61" s="37" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="C61" s="37"/>
       <c r="D61" s="48" t="inlineStr">
         <is>
-          <t>Có nhắc mốc thanh toán; thiếu nhắc gia hạn/kết thúc hợp đồng.</t>
+          <t xml:space="preserve">Email tự động theo ngày nhắc riêng; có xem trước, lịch sử gửi và mẫu tại /admin/email-templates.</t>
         </is>
       </c>
       <c r="E61" s="49"/>

</xml_diff>

<commit_message>
Refresh NICON delivery status evidence
Replace stale Concept and lead-conversion statuses with source-backed
Implemented labels. Record reminder delivery boundaries and remaining
BOQ, finance, reporting, and KPI gaps with code and test references.

Preserve requirements, estimates, formulas, and unrelated workbook parts.
Validate workbook integrity and rendered changes without runtime tests.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -2503,7 +2503,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d.m"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="24">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -2611,8 +2611,32 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="23">
+  <fills count="26">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2745,6 +2769,21 @@
         <bgColor rgb="FF00FFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA4C2F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF79646"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="8">
     <border/>
@@ -2823,10 +2862,11 @@
       </bottom>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="116">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3100,6 +3140,40 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="0" shrinkToFit="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3431,7 +3505,7 @@
     <col customWidth="1" min="5" max="5" width="85.43"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.75" customHeight="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3441,9 +3515,9 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ghi chú — đối chiếu source d884b3c6, 20/10/2026; không xác nhận host/UAT</t>
+      <c r="D1" s="104" t="inlineStr">
+        <is>
+          <t>Ghi chú — đối chiếu source 7813bc5d, 21/10/2026; rà soát source/test hiện có, không chạy lại test, không xác nhận host/UAT</t>
         </is>
       </c>
       <c r="E1" s="2"/>
@@ -4410,7 +4484,7 @@
       <c r="D60" s="48"/>
       <c r="E60" s="49"/>
     </row>
-    <row r="61">
+    <row r="61" ht="78" customHeight="1">
       <c r="A61" s="44" t="s">
         <v>279</v>
       </c>
@@ -4420,14 +4494,14 @@
         </is>
       </c>
       <c r="C61" s="37"/>
-      <c r="D61" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Email tự động theo ngày nhắc riêng; có xem trước, lịch sử gửi và mẫu tại /admin/email-templates.</t>
+      <c r="D61" s="105" t="inlineStr">
+        <is>
+          <t>Upstream: chọn Renewal/End, ngày Việt Nam, người liên hệ → preview → xác nhận. Worker 5 phút/lần; mẫu tại /admin/email-templates; ghi chăm sóc sau SMTP. ContractReminderService/Worker; ContractRemindersTests; contract-reminder-email.spec.ts. Không tự gia hạn/đóng HĐ; Sending/NeedsReview cần đối soát, không tự retry.</t>
         </is>
       </c>
       <c r="E61" s="49"/>
     </row>
-    <row r="62">
+    <row r="62" ht="61" customHeight="1">
       <c r="A62" s="44" t="s">
         <v>283</v>
       </c>
@@ -4437,14 +4511,14 @@
         </is>
       </c>
       <c r="C62" s="37"/>
-      <c r="D62" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Timeline riêng theo HĐ; phân quyền, phân trang, retry; có lịch sử thì khóa đổi chiều.</t>
+      <c r="D62" s="105" t="inlineStr">
+        <is>
+          <t>Lịch sử chăm sóc riêng theo HĐ. Khóa đổi chiều sau lịch sử hoặc lần bắt đầu gửi email (AttemptedAt), kể cả SMTP chưa rõ kết quả. ContractService; ContractCareActivitiesTests; ContractRemindersTests.</t>
         </is>
       </c>
       <c r="E62" s="49"/>
     </row>
-    <row r="63">
+    <row r="63" ht="44" customHeight="1">
       <c r="A63" s="44" t="s">
         <v>290</v>
       </c>
@@ -4454,7 +4528,11 @@
         </is>
       </c>
       <c r="C63" s="37"/>
-      <c r="D63" s="48"/>
+      <c r="D63" s="105" t="inlineStr">
+        <is>
+          <t>Chưa thấy workflow tái ký/liên kết HĐ kế tiếp trong ContractService/ContractDetail. Email Renewal chỉ nhắc khách, không tạo/gia hạn HĐ mới.</t>
+        </is>
+      </c>
       <c r="E63" s="49"/>
     </row>
     <row r="64">
@@ -4501,36 +4579,36 @@
       <c r="D67" s="44"/>
       <c r="E67" s="39"/>
     </row>
-    <row r="68">
+    <row r="68" ht="61" customHeight="1">
       <c r="A68" s="40" t="s">
         <v>314</v>
       </c>
-      <c r="B68" s="37" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="B68" s="106" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="C68" s="37"/>
-      <c r="D68" s="44" t="inlineStr">
-        <is>
-          <t>Có lưu file thiết kế; thiếu quản lý/xem mô hình 3D chuyên dụng.</t>
+      <c r="D68" s="107" t="inlineStr">
+        <is>
+          <t>Quản lý file Model3D theo phương án/revision; tải bản gốc, ảnh/PDF có preview. ConceptDossierService.AddArtifactAsync; ConceptDossierPanel; admin-concept-dossier.spec.ts. Theo Nicon-QLVH §4, trình xem 3D chuyên dụng không là điều kiện hoàn thành.</t>
         </is>
       </c>
       <c r="E68" s="39"/>
     </row>
-    <row r="69">
+    <row r="69" ht="61" customHeight="1">
       <c r="A69" s="40" t="s">
         <v>317</v>
       </c>
-      <c r="B69" s="37" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="B69" s="106" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="C69" s="37"/>
-      <c r="D69" s="44" t="inlineStr">
-        <is>
-          <t>Có lưu bản vẽ Concept; thiếu quản lý mặt bằng công năng theo cấu trúc riêng.</t>
+      <c r="D69" s="107" t="inlineStr">
+        <is>
+          <t>FloorPlan có FloorLabel bắt buộc, tách SiteRoofPlan/Section; file đúng phương án/revision, sửa liên kết khi nháp. ConceptDossierService; ConceptDossierPanel; DesignReviewsControllerTests.ConceptDraft_CanCorrectFileAndWaiver_ButFrozenRevisionCannotChange.</t>
         </is>
       </c>
       <c r="E69" s="39"/>
@@ -4548,53 +4626,53 @@
       <c r="D70" s="44"/>
       <c r="E70" s="39"/>
     </row>
-    <row r="71">
+    <row r="71" ht="78" customHeight="1">
       <c r="A71" s="40" t="s">
         <v>326</v>
       </c>
-      <c r="B71" s="37" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="B71" s="106" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="C71" s="37"/>
-      <c r="D71" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có bình luận nội bộ gắn từng file và ghi nhận ý kiến khách; chưa có thread/markup trực tiếp của khách.</t>
+      <c r="D71" s="107" t="inlineStr">
+        <is>
+          <t>Ý kiến khách: nguyên văn, tên, kênh, thời điểm, nguồn bằng chứng, file; phản hồi/kết quả một lần. ConceptDossierService.AddFeedbackAsync/RespondAsync; ConceptDossierPanel; DesignReviewsControllerTests.ConceptDecision_RequiresSignedAcceptanceAndPreservesRejectedState. Markup đồ họa vẫn là Target riêng.</t>
         </is>
       </c>
       <c r="E71" s="39"/>
     </row>
-    <row r="72">
+    <row r="72" ht="78" customHeight="1">
       <c r="A72" s="40" t="s">
         <v>330</v>
       </c>
-      <c r="B72" s="37" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="B72" s="106" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="C72" s="37"/>
-      <c r="D72" s="44" t="inlineStr">
-        <is>
-          <t>Có nhiều phương án Concept; thiếu revision/version của cùng một phương án.</t>
+      <c r="D72" s="107" t="inlineStr">
+        <is>
+          <t>ConceptRevision R00/R01... theo cùng phương án; bản đã trình bất biến; revision mới sau yêu cầu sửa/từ chối. ConceptDossierService.CreateRevisionAsync; ConceptDossierPanel; DesignReviewsControllerTests.ClientChanges_CreateR01_PreservesR00AndRejectsIncompleteSubmission; ConceptDossierConcurrencyTests.</t>
         </is>
       </c>
       <c r="E72" s="39"/>
     </row>
-    <row r="73">
+    <row r="73" ht="78" customHeight="1">
       <c r="A73" s="40" t="s">
         <v>334</v>
       </c>
-      <c r="B73" s="37" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="B73" s="106" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="C73" s="37"/>
-      <c r="D73" s="44" t="inlineStr">
-        <is>
-          <t>Có gate quyết định khách hàng; thiếu ký/chốt trực tiếp trên portal khách hàng.</t>
+      <c r="D73" s="107" t="inlineStr">
+        <is>
+          <t>Trình nội bộ → ghi nhận trình khách → ClientApproved kèm TK-M03 đã ký, người/ngày ký → chốt một phương án và mở Basic Design. ConceptOptionService; DesignReviewService; DesignReviewsTab; ConceptFinalizationPersistenceTests; ConceptOptionServiceTests. Không yêu cầu portal khách hàng theo Nicon-QLVH §4.</t>
         </is>
       </c>
       <c r="E73" s="39"/>
@@ -11351,27 +11429,38 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="218.0"/>
     <col customWidth="1" min="2" max="2" width="15.14"/>
+    <col min="3" max="3" width="104" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="16" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="18" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
+      <c r="C1" s="108" t="inlineStr">
+        <is>
+          <t>Đối chiếu source 7813bc5d, 21/10/2026; không chạy lại test, không xác nhận host/UAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="61" customHeight="1">
       <c r="A2" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
+      <c r="B2" s="109" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="C2" s="110" t="inlineStr">
+        <is>
+          <t>LeadService cho phép TaxId null; Leads.tsx không bắt MST khi convert. LeadsControllerTests.Convert_CompanyLeadWithoutTaxId_PreservesCustomerAndOpportunityLinks. Điều kiện pháp lý khi ký HĐ là gate khác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
       <c r="A3" s="19" t="s">
         <v>24</v>
       </c>
@@ -11380,8 +11469,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
+      <c r="C3" s="110" t="inlineStr">
+        <is>
+          <t>QuoteService cho phép cơ hội Won chưa có WonQuoteId tạo báo giá; chặn khi đã có báo giá thắng. QuotesControllerTests; CrmBusinessPipelineTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="61" customHeight="1">
       <c r="A4" s="19" t="s">
         <v>27</v>
       </c>
@@ -11390,8 +11484,13 @@
           <t xml:space="preserve">Partial</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
+      <c r="C4" s="110" t="inlineStr">
+        <is>
+          <t>Có BOQ catalog/revision, nhập cấu hình, preview và validation (BoqConfiguredWorkbookService, ConfiguredBoqControllerTests). Yêu cầu lỗi gốc chưa có bước tái hiện cụ thể, chưa xác nhận UAT; giữ Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
       <c r="A5" s="19" t="s">
         <v>29</v>
       </c>
@@ -11400,8 +11499,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
+      <c r="C5" s="110" t="inlineStr">
+        <is>
+          <t>CapabilityDocumentsController/CapabilityDocumentService và CapabilityDocuments.tsx có CRUD/phân quyền; CapabilityDocumentsControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
       <c r="A6" s="19" t="s">
         <v>31</v>
       </c>
@@ -11410,8 +11514,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
+      <c r="C6" s="110" t="inlineStr">
+        <is>
+          <t>ContractService tự sinh số khi để trống, cho nhập số riêng/kiểm tra trùng; Contracts.tsx có preview gợi ý. ContractsControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
       <c r="A7" s="19" t="s">
         <v>34</v>
       </c>
@@ -11420,8 +11529,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
+      <c r="C7" s="110" t="inlineStr">
+        <is>
+          <t>ContractDetail có hướng dẫn VO qua i18n; ContractAppendixService xử lý phát sinh/duyệt. Không đổi trạng thái đã có.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="19" t="s">
         <v>40</v>
       </c>
@@ -11430,8 +11544,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
+      <c r="C8" s="110" t="inlineStr">
+        <is>
+          <t>ContractDetail/ContractCareActivities hiển thị event qua i18n; seed bản dịch 4 ngôn ngữ. Giữ Implemented theo source; chưa chạy lại UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="19" t="s">
         <v>43</v>
       </c>
@@ -11440,8 +11559,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="22.5" customHeight="1">
+      <c r="C9" s="110" t="inlineStr">
+        <is>
+          <t>Design schedule task có assignee/approver/CC và dependency, cho việc không phụ thuộc chạy song song. DetailDesignScheduleService; DetailDesignScheduleControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="61" customHeight="1">
       <c r="A10" s="19" t="s">
         <v>46</v>
       </c>
@@ -11450,8 +11574,13 @@
           <t xml:space="preserve">Partial</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="22.5" customHeight="1">
+      <c r="C10" s="110" t="inlineStr">
+        <is>
+          <t>Có mẫu BOQ NICON trong docs/Nicon/BOQ và nhập preview/mapping danh mục. Chưa có schema tổng quát giữ hierarchy/provenance/công thức cho mọi workbook; giữ Partial. BoqCatalogWorkbookService; Nicon-QLVH §7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
       <c r="A11" s="19" t="s">
         <v>49</v>
       </c>
@@ -11460,8 +11589,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
+      <c r="C11" s="110" t="inlineStr">
+        <is>
+          <t>DesignProjectTeamTab và ProjectTeamService quản lý thành viên trên Operational Project; OperationalProjectTeamControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
       <c r="A12" s="19" t="s">
         <v>51</v>
       </c>
@@ -11470,8 +11604,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="22.5" customHeight="1">
+      <c r="C12" s="110" t="inlineStr">
+        <is>
+          <t>Có deadline/checklist đấu thầu và lịch các giai đoạn thiết kế. TenderService; DetailDesignScheduleService; TendersControllerTests; DetailDesignScheduleControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="44" customHeight="1">
       <c r="A13" s="19" t="s">
         <v>56</v>
       </c>
@@ -11480,8 +11619,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="22.5" customHeight="1">
+      <c r="C13" s="110" t="inlineStr">
+        <is>
+          <t>DesignScheduleTab/Timeline có phase/task, kế hoạch/thực tế/trọng số. DetailDesignScheduleControllerTests. Nhập .mpp đầy đủ vẫn là Target riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="61" customHeight="1">
       <c r="A14" s="19" t="s">
         <v>60</v>
       </c>
@@ -11490,8 +11634,13 @@
           <t xml:space="preserve">Partial</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="22.5" customHeight="1">
+      <c r="C14" s="110" t="inlineStr">
+        <is>
+          <t>Work package/design/tender có lịch và dependency. Chưa có SLA mọi công tác và quy tắc Lead 1 tuần được xác nhận/cấu hình; giữ Partial. DepartmentWorkPackageService; DetailDesignScheduleService.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
       <c r="A15" s="19" t="s">
         <v>63</v>
       </c>
@@ -11500,8 +11649,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="22.5" customHeight="1">
+      <c r="C15" s="110" t="inlineStr">
+        <is>
+          <t>Nhãn giao diện Detail Design qua i18n; tên entity/API ShopDrawing giữ tương thích. ShopDrawingTab; ShopDrawingsControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
       <c r="A16" s="19" t="s">
         <v>67</v>
       </c>
@@ -11510,8 +11664,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="22.5" customHeight="1">
+      <c r="C16" s="110" t="inlineStr">
+        <is>
+          <t>DesignProjectTeamTab/DesignScheduleTab có giao việc/duyệt; KpiService đọc tiến độ thiết kế. DetailDesignScheduleControllerTests; KpiControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
       <c r="A17" s="19" t="s">
         <v>69</v>
       </c>
@@ -11520,8 +11679,13 @@
           <t xml:space="preserve">Partial</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
+      <c r="C17" s="110" t="inlineStr">
+        <is>
+          <t>ProjectDocumentService/ProjectDriveSyncService có durable sync nhiều module; chưa chứng minh tất cả đường upload/Drive NICON thật. Nicon-QLVH §9; ProjectDocumentServiceTests. Giữ Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="61" customHeight="1">
       <c r="A18" s="19" t="s">
         <v>74</v>
       </c>
@@ -11530,8 +11694,13 @@
           <t xml:space="preserve">Partial</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
+      <c r="C18" s="110" t="inlineStr">
+        <is>
+          <t>OperationalProjectService/ProjectAccessService và báo cáo có scope dự án; aggregate thi công cũ còn DesignProjectId. Migration hợp nhất cần backfill/rehearsal/rollback; giữ Partial theo Nicon-QLVH §6.6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1">
       <c r="A19" s="19" t="s">
         <v>77</v>
       </c>
@@ -11540,8 +11709,13 @@
           <t xml:space="preserve">Partial</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
+      <c r="C19" s="110" t="inlineStr">
+        <is>
+          <t>ProjectReportService có báo cáo dự án và XLSX/PDF, nguồn CM. actualCashflow/profitAndLoss/inventory chưa khả dụng trong báo cáo chung; ProjectReportsControllerTests. Giữ Partial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
       <c r="A20" s="19" t="s">
         <v>82</v>
       </c>
@@ -11550,8 +11724,13 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
+      <c r="C20" s="110" t="inlineStr">
+        <is>
+          <t>Customer → nhiều OperationalProject; Opportunity có CustomerId/OperationalProjectId. OperationalProjectService; OpportunityService; OperationalProjectsControllerTests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
       <c r="A21" s="19" t="s">
         <v>86</v>
       </c>
@@ -11560,14 +11739,24 @@
           <t xml:space="preserve">Implemented</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
+      <c r="C21" s="110" t="inlineStr">
+        <is>
+          <t>DesignProject thuộc OperationalProject, bắt đầu trước HĐ đã ký. DesignProjectService; DesignProjectsControllerTests; Nicon-QLVH §4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
       <c r="A22" s="19" t="s">
         <v>88</v>
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="C22" s="110" t="inlineStr">
+        <is>
+          <t>Có application_developer.md, user_guide.md, users-rbac.md và tài khoản seed. Đây là hướng dẫn trong repo, không xác nhận đã bàn giao host/tài khoản thật.</t>
         </is>
       </c>
     </row>
@@ -11596,7 +11785,7 @@
     <col customWidth="1" min="8" max="8" width="18.43"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
@@ -11612,9 +11801,9 @@
       <c r="E1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ghi chú — đối chiếu source d884b3c6, 20/10/2026</t>
+      <c r="F1" s="111" t="inlineStr">
+        <is>
+          <t>Ghi chú — đối chiếu source 7813bc5d, 21/10/2026; không chạy lại test, không xác nhận host/UAT</t>
         </is>
       </c>
       <c r="G1" s="12" t="s">
@@ -12058,7 +12247,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="95" customHeight="1">
       <c r="A21" s="17">
         <v>20.0</v>
       </c>
@@ -12070,9 +12259,9 @@
       <c r="E21" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="F21" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có tiến độ theo HĐ, nguồn Lead và timeline chăm sóc riêng; có lịch sử thì khóa đổi chiều.</t>
+      <c r="F21" s="114" t="inlineStr">
+        <is>
+          <t>Có nguồn Lead, tiến độ theo HĐ, phụ lục/mốc/file, chăm sóc riêng và email nhắc tự động. ContractExecutionProgressService; ContractReminderService; ContractSourceLeadsTests; ContractRemindersTests. Khóa đổi chiều từ lần bắt đầu gửi; Dự án vận hành là gốc nghiệp vụ.</t>
         </is>
       </c>
       <c r="G21" s="17"/>
@@ -12198,7 +12387,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="36" customHeight="1">
+    <row r="27" ht="112" customHeight="1">
       <c r="A27" s="17">
         <v>26.0</v>
       </c>
@@ -12210,15 +12399,15 @@
       <c r="E27" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="F27" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có review nội bộ gắn file và ghi nhận quyết định khách; chưa có portal ký/markup trực tiếp.</t>
+      <c r="F27" s="113" t="inlineStr">
+        <is>
+          <t>Concept dossier: file theo loại/tầng, revision bất biến, feedback và kết quả xử lý, duyệt TK-M03 đã ký. ConceptDossierService/Panel; DesignReviewsControllerTests; ConceptFinalizationPersistenceTests; admin-concept-dossier.spec.ts. Portal/markup không thuộc gate hoàn thành đã xác nhận.</t>
         </is>
       </c>
       <c r="G27" s="17"/>
-      <c r="H27" s="25" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="H27" s="112" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
     </row>
@@ -13156,7 +13345,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="36" customHeight="1">
+    <row r="68" ht="78" customHeight="1">
       <c r="A68" s="17">
         <v>67.0</v>
       </c>
@@ -13168,9 +13357,9 @@
       <c r="E68" s="23" t="s">
         <v>381</v>
       </c>
-      <c r="F68" s="103" t="inlineStr">
-        <is>
-          <t>Create/Edit form | Thiếu import đa sheet giữ hierarchy, provenance, công thức và tổng hợp đối soát.</t>
+      <c r="F68" s="113" t="inlineStr">
+        <is>
+          <t>Có BOQ draft/revision và nhập danh mục cấu hình. Còn thiếu import Execution BOQ đa sheet giữ hierarchy/provenance từng dòng, baseline và đối soát công thức. BoqCatalogWorkbookService; ProcurementService; Nicon-QLVH §7.</t>
         </is>
       </c>
       <c r="G68" s="17"/>
@@ -13574,7 +13763,7 @@
         </is>
       </c>
     </row>
-    <row r="86">
+    <row r="86" ht="78" customHeight="1">
       <c r="A86" s="17">
         <v>85.0</v>
       </c>
@@ -13588,8 +13777,10 @@
       <c r="E86" s="23" t="s">
         <v>488</v>
       </c>
-      <c r="F86" s="17" t="s">
-        <v>489</v>
+      <c r="F86" s="114" t="inlineStr">
+        <is>
+          <t>Target — FinanceService có Payment Request/period/correction; ProjectReportService khai báo actualCashflow unavailable. Chưa có sổ thực thu–chi/forecast tổng hợp. Không coi Paid milestone là ledger.</t>
+        </is>
       </c>
       <c r="G86" s="17"/>
       <c r="H86" s="25" t="inlineStr">
@@ -13598,7 +13789,7 @@
         </is>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="61" customHeight="1">
       <c r="A87" s="17">
         <v>86.0</v>
       </c>
@@ -13612,8 +13803,10 @@
       <c r="E87" s="23" t="s">
         <v>493</v>
       </c>
-      <c r="F87" s="17" t="s">
-        <v>494</v>
+      <c r="F87" s="114" t="inlineStr">
+        <is>
+          <t>Target — ProjectReportService khai báo profitAndLoss/actualRevenue/actualExpenditure unavailable; chưa có nguồn ledger doanh thu/chi phí để tính P&amp;L.</t>
+        </is>
       </c>
       <c r="G87" s="17"/>
       <c r="H87" s="25" t="inlineStr">
@@ -13730,7 +13923,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="36" customHeight="1">
+    <row r="92" ht="78" customHeight="1">
       <c r="A92" s="17">
         <v>91.0</v>
       </c>
@@ -13744,9 +13937,9 @@
       <c r="E92" s="77" t="s">
         <v>289</v>
       </c>
-      <c r="F92" s="103" t="inlineStr">
-        <is>
-          <t>Setting + CRUD | Có cấu hình 6 nhóm KPI; thiếu framework đủ 11 vị trí NICON.</t>
+      <c r="F92" s="113" t="inlineStr">
+        <is>
+          <t>KpiService/KpiConfiguration: 19 metric, 6 nhóm scorecard; có trọng số/target/ngưỡng. Còn thiếu framework đủ 11 vị trí và nguồn HR/Admin. KpiControllerTests; Nicon-QLVH §10.</t>
         </is>
       </c>
       <c r="G92" s="78" t="s">
@@ -13758,7 +13951,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="36" customHeight="1">
+    <row r="93" ht="61" customHeight="1">
       <c r="A93" s="17">
         <v>92.0</v>
       </c>
@@ -13770,9 +13963,9 @@
       <c r="E93" s="77" t="s">
         <v>298</v>
       </c>
-      <c r="F93" s="103" t="inlineStr">
-        <is>
-          <t>Integration/rule config | Có mapping nguồn cho 19 chỉ số; thiếu nguồn/rule cho các vị trí còn lại.</t>
+      <c r="F93" s="113" t="inlineStr">
+        <is>
+          <t>KpiService có mapping 19 metric và MissingData; chưa đủ nguồn budget/S-Curve/tuyển dụng cho 11 vị trí. Nicon-QLVH §10; application_developer §7.19.</t>
         </is>
       </c>
       <c r="G93" s="79">
@@ -13784,7 +13977,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="36" customHeight="1">
+    <row r="94" ht="78" customHeight="1">
       <c r="A94" s="17">
         <v>93.0</v>
       </c>
@@ -13796,9 +13989,9 @@
       <c r="E94" s="77" t="s">
         <v>306</v>
       </c>
-      <c r="F94" s="103" t="inlineStr">
-        <is>
-          <t>Backend service | Có engine và khóa kỳ; thiếu chỉ số đầy đủ cho 11 vị trí.</t>
+      <c r="F94" s="113" t="inlineStr">
+        <is>
+          <t>Có tính ngày 01:00 giờ Việt Nam, tính thủ công, lịch sử và khóa snapshot; vẫn Partial theo phạm vi 11 vị trí. KpiCalculationBackgroundService; KpiService; KpiControllerTests.</t>
         </is>
       </c>
       <c r="G94" s="78" t="s">
@@ -13836,7 +14029,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="36" customHeight="1">
+    <row r="96" ht="61" customHeight="1">
       <c r="A96" s="17">
         <v>95.0</v>
       </c>
@@ -13848,9 +14041,9 @@
       <c r="E96" s="77" t="s">
         <v>322</v>
       </c>
-      <c r="F96" s="103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có CSV KPI theo nhân viên/kỳ; chưa có Google Sheets/PDF và lưu tự động lên Drive.</t>
+      <c r="F96" s="113" t="inlineStr">
+        <is>
+          <t>KpiController.Export hiện trả CSV theo nhân viên/kỳ. Chưa có Google Sheets/PDF, export toàn công ty và tự lưu Drive theo yêu cầu. Giữ Partial.</t>
         </is>
       </c>
       <c r="G96" s="79">
@@ -13998,7 +14191,7 @@
         </is>
       </c>
     </row>
-    <row r="102">
+    <row r="102" ht="61" customHeight="1">
       <c r="A102" s="17">
         <v>101.0</v>
       </c>
@@ -14014,8 +14207,10 @@
       <c r="E102" s="23" t="s">
         <v>543</v>
       </c>
-      <c r="F102" s="88" t="s">
-        <v>4</v>
+      <c r="F102" s="115" t="inlineStr">
+        <is>
+          <t>Chưa thấy global search/saved filters dùng chung; các module có tìm kiếm/lọc riêng. Giữ Target cho đúng phạm vi yêu cầu.</t>
+        </is>
       </c>
       <c r="G102" s="17"/>
       <c r="H102" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Add contract renewal and expansion workflow
Track immutable source contracts for renewal and expansion pursuits.
Create independent draft contracts directly or through opportunities and
approved quotes, with scoped access and retry-safe creation.

Preserve provenance during updates and permanent deletion. Add demo data,
translations, customer guidance, and the verified workbook delivery status.
Cover lifecycle, authorization, concurrency, and responsive live flows.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4518,19 +4518,19 @@
       </c>
       <c r="E62" s="49"/>
     </row>
-    <row r="63" ht="44" customHeight="1">
+    <row r="63" ht="95" customHeight="1">
       <c r="A63" s="44" t="s">
         <v>290</v>
       </c>
-      <c r="B63" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Target</t>
+      <c r="B63" s="106" t="inlineStr">
+        <is>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="C63" s="37"/>
       <c r="D63" s="105" t="inlineStr">
         <is>
-          <t>Chưa thấy workflow tái ký/liên kết HĐ kế tiếp trong ContractService/ContractDetail. Email Renewal chỉ nhắc khách, không tạo/gia hạn HĐ mới.</t>
+          <t>Upstream đã ký → Renewal/Expansion → HĐ Draft độc lập hoặc Cơ hội đàm phán/Won/Lost. Nguồn/mục đích/lý do bất biến; cùng khách, chọn Dự án theo quyền; hỗ trợ tạo trực tiếp/Báo giá duyệt, truy vết hai chiều, idempotency và chặn xóa lịch sử. ContractContinuationRules; ContractContinuationsTests; contract-continuations.spec.ts (390/768px). Quy tắc theo chỉ đạo người dùng 22/10/2026; không tự đổi HĐ cũ. Không xác nhận production/UAT.</t>
         </is>
       </c>
       <c r="E63" s="49"/>

</xml_diff>

<commit_message>
Fix contract continuation form recovery
Clear continuation context when cancelling so ordinary creation keeps
its customer editable. Show source-loading failures in the open form and
retry source or reference data without discarding entered deal terms.

Refresh stale source versions safely, focus validation errors, and use a
multiline reason field. Expand live browser coverage for cancellation,
keyboard access, concurrency recovery, responsive layouts, and languages.
Update the workbook evidence and operating guidance after verification.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4518,7 +4518,7 @@
       </c>
       <c r="E62" s="49"/>
     </row>
-    <row r="63" ht="95" customHeight="1">
+    <row r="63" ht="112" customHeight="1">
       <c r="A63" s="44" t="s">
         <v>290</v>
       </c>
@@ -4530,7 +4530,7 @@
       <c r="C63" s="37"/>
       <c r="D63" s="105" t="inlineStr">
         <is>
-          <t>Upstream đã ký → Renewal/Expansion → HĐ Draft độc lập hoặc Cơ hội đàm phán/Won/Lost. Nguồn/mục đích/lý do bất biến; cùng khách, chọn Dự án theo quyền; hỗ trợ tạo trực tiếp/Báo giá duyệt, truy vết hai chiều, idempotency và chặn xóa lịch sử. ContractContinuationRules; ContractContinuationsTests; contract-continuations.spec.ts (390/768px). Quy tắc theo chỉ đạo người dùng 22/10/2026; không tự đổi HĐ cũ. Không xác nhận production/UAT.</t>
+          <t>Upstream đã ký → Renewal/Expansion → HĐ Draft riêng hoặc Cơ hội đàm phán/Won/Lost; truy vết nguồn bất biến, phân quyền, idempotency, chặn xóa lịch sử. Review UI/UX: hủy form rồi tạo độc lập; lỗi tải nguồn/thử lại; cập nhật nguồn khi xung đột mà giữ nội dung; lý do nhiều dòng, focus lỗi. Regression: 154 unit, 120 integration; E2E 390/768/1440px, bàn phím, vi/en/zh/ja. Không tự đổi HĐ cũ. Theo chỉ đạo người dùng 22/10/2026. Không xác nhận production/UAT; không hỗ trợ mở trang chưa tải khi hoàn toàn offline.</t>
         </is>
       </c>
       <c r="E63" s="49"/>

</xml_diff>

<commit_message>
Record legal checklist delivery progress
Update the task workbook with delivered legal template, concurrency,
closed-package and predecessor behavior verified on 75f41b6d.

Keep the complete permit matrix scope Partial and identify the NICON
owners and decisions needed for project applicability and ISO control.
Preserve unrelated workbook cells, formulas, validations and sheets.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -2866,7 +2866,7 @@
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="121">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -3174,6 +3174,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5154,7 +5169,7 @@
       <c r="D110" s="44"/>
       <c r="E110" s="39"/>
     </row>
-    <row r="111">
+    <row r="111" ht="70" customHeight="1">
       <c r="A111" s="40" t="s">
         <v>515</v>
       </c>
@@ -5164,7 +5179,11 @@
         </is>
       </c>
       <c r="C111" s="37"/>
-      <c r="D111" s="48"/>
+      <c r="D111" s="116" t="inlineStr">
+        <is>
+          <t>22/10/2026, 75f41b6d: Implemented phần setup PM/Admin. Chặn thêm permit/task vào gói Completed/Cancelled. Hợp đồng khác chỉ dùng lại gói Completed có snapshot khi không sửa hồ sơ. Regression integration đã pass.</t>
+        </is>
+      </c>
       <c r="E111" s="49"/>
     </row>
     <row r="112">
@@ -5180,7 +5199,7 @@
       <c r="D112" s="48"/>
       <c r="E112" s="49"/>
     </row>
-    <row r="113">
+    <row r="113" ht="95" customHeight="1">
       <c r="A113" s="40" t="s">
         <v>518</v>
       </c>
@@ -5190,9 +5209,9 @@
         </is>
       </c>
       <c r="C113" s="37"/>
-      <c r="D113" s="80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Có checklist theo Dự án; CM/NICON chưa duyệt template bắt buộc theo loại/quy mô công trình.</t>
+      <c r="D113" s="117" t="inlineStr">
+        <is>
+          <t>22/10/2026, 75f41b6d: Implemented phần mềm soạn mẫu 4 ngôn ngữ, duyệt độc lập, phiên bản/retire, snapshot dự án và kiểm tra mục bắt buộc. Toàn phạm vi vẫn Partial. Open decision Q-09 — CM/NICON chốt ma trận theo loại/quy mô, miễn/ngoại lệ và permit chặn từng mốc khởi công. PM hiện chọn mẫu thủ công. GĐ/ĐDCL/TKISO xác nhận ủy quyền phát hành điện tử, thu hồi, lưu/hủy hồ sơ ISO.</t>
         </is>
       </c>
       <c r="E113" s="81"/>
@@ -5236,7 +5255,7 @@
       <c r="D116" s="84"/>
       <c r="E116" s="83"/>
     </row>
-    <row r="117">
+    <row r="117" ht="70" customHeight="1">
       <c r="A117" s="40" t="s">
         <v>524</v>
       </c>
@@ -5246,7 +5265,11 @@
         </is>
       </c>
       <c r="C117" s="37"/>
-      <c r="D117" s="84"/>
+      <c r="D117" s="118" t="inlineStr">
+        <is>
+          <t>22/10/2026, 75f41b6d: Implemented phân công thành viên dự án, người duyệt độc lập, lịch và predecessor. Permit đã có task cùng dự án làm predecessor cho việc mới. Token cũ bị từ chối 409. Đổi lịch/chủ trì lưu history trước/sau và actor. Regression integration và live E2E đã pass.</t>
+        </is>
+      </c>
       <c r="E117" s="83"/>
     </row>
     <row r="118">
@@ -12691,7 +12714,7 @@
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="70" customHeight="1">
       <c r="A40" s="17">
         <v>39.0</v>
       </c>
@@ -12707,8 +12730,10 @@
       <c r="E40" s="23" t="s">
         <v>238</v>
       </c>
-      <c r="F40" s="17" t="s">
-        <v>26</v>
+      <c r="F40" s="119" t="inlineStr">
+        <is>
+          <t>22/10/2026, 75f41b6d: Implemented danh sách permit theo dự án và quản lý mẫu. Có mẫu 4 ngôn ngữ, duyệt độc lập, phiên bản/retire. Demo chỉ có mẫu nháp. CM/NICON cần duyệt nội dung mẫu sản xuất theo Q-09.</t>
+        </is>
       </c>
       <c r="G40" s="17"/>
       <c r="H40" s="25" t="inlineStr">
@@ -12717,7 +12742,7 @@
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="80" customHeight="1">
       <c r="A41" s="17">
         <v>40.0</v>
       </c>
@@ -12729,8 +12754,10 @@
       <c r="E41" s="23" t="s">
         <v>243</v>
       </c>
-      <c r="F41" s="17" t="s">
-        <v>33</v>
+      <c r="F41" s="119" t="inlineStr">
+        <is>
+          <t>22/10/2026, 75f41b6d: Implemented setup bằng mẫu Published, snapshot và mục bắt buộc. Chặn sửa gói đóng, stale request trả 409, lưu history lịch/chủ trì. GPXD hiện hữu làm predecessor cho PCCC mới. Checklist tự khớp loại/quy mô còn Partial: CM/NICON chốt Q-09, ngoại lệ và gate khởi công.</t>
+        </is>
       </c>
       <c r="G41" s="17"/>
       <c r="H41" s="25" t="inlineStr">
@@ -12739,7 +12766,7 @@
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="70" customHeight="1">
       <c r="A42" s="17">
         <v>41.0</v>
       </c>
@@ -12751,8 +12778,10 @@
       <c r="E42" s="23" t="s">
         <v>245</v>
       </c>
-      <c r="F42" s="17" t="s">
-        <v>38</v>
+      <c r="F42" s="119" t="inlineStr">
+        <is>
+          <t>22/10/2026, 75f41b6d: Giữ Implemented hồ sơ/trạng thái/timeline. Đã xác nhận phạm vi Legal bằng 21 unit, 25 integration, 2 live E2E trên Compose và 2 UI mock riêng. Live E2E gồm mobile/tablet và phục hồi stale edit. Không xác nhận host/UAT NICON.</t>
+        </is>
       </c>
       <c r="G42" s="17"/>
       <c r="H42" s="25" t="inlineStr">
@@ -14247,7 +14276,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="36" customHeight="1">
+    <row r="104" ht="70" customHeight="1">
       <c r="A104" s="17">
         <v>103.0</v>
       </c>
@@ -14263,9 +14292,9 @@
       <c r="E104" s="23" t="s">
         <v>552</v>
       </c>
-      <c r="F104" s="103" t="inlineStr">
-        <is>
-          <t>Chức năng chung | Có master data dùng chung; thiếu template/checklist theo dự án và approval matrix NICON.</t>
+      <c r="F104" s="120" t="inlineStr">
+        <is>
+          <t>22/10/2026, 75f41b6d: Có master data và engine mẫu checklist Pháp lý 4 ngôn ngữ, duyệt độc lập, phiên bản, snapshot dự án. Giữ Partial: CM/NICON chốt ma trận theo loại/quy mô, miễn/ngoại lệ, gate áp dụng và approval matrix chính thức. GĐ/ĐDCL/TKISO xác nhận ủy quyền phát hành/lưu hủy ISO.</t>
         </is>
       </c>
       <c r="G104" s="17"/>

</xml_diff>

<commit_message>
Mark construction drawing links implemented
Update the task plan after verifying the released IFC/WBS workflow
and passing validation for commit 491f0038 in PR #301. Mark Nicon!B89
Implemented and replace the obsolete missing-link note at D89.

Keep every other cell, formula, format, sheet visibility and drawing
unchanged. Record that the PR is open and host/UAT is not confirmed.
</commit_message>
<xml_diff>
--- a/docs/Nicon_BreakTask_v1.xlsx
+++ b/docs/Nicon_BreakTask_v1.xlsx
@@ -4870,13 +4870,13 @@
       </c>
       <c r="B89" s="37" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="C89" s="37"/>
       <c r="D89" s="44" t="inlineStr">
         <is>
-          <t>Có hồ sơ Shop Drawing theo bộ môn; thiếu liên kết bản vẽ đến WBS/hạng mục thi công ổn định.</t>
+          <t>22/10/2026, 491f0038. IFC–WBS có API/UI, test đạt. PR #301 mở; chưa xác nhận host/UAT.</t>
         </is>
       </c>
       <c r="E89" s="39"/>

</xml_diff>